<commit_message>
Add a new fallback for DHL suggestions based on regional proximity
Introduces a `region_any_km` fallback to `dhlAutoTableSelector.ts`, updates UI components (`MissionFinancialModal.tsx`) to display this new level with amber styling, and modifies the `dhl-antes-depois.ts` script to correctly count and report on this new matching strategy.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: e7487dfc-a007-4c28-82b0-fb98492115a4
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 01991df6-ff3e-4ab5-958d-d54e8eb57bcc
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/bfb67e20-5400-4562-9712-6800cf5333e4/e7487dfc-a007-4c28-82b0-fb98492115a4/5KMGFOL
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/exports/dhl-antes-depois.xlsx
+++ b/exports/dhl-antes-depois.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -443,39 +443,63 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SEM sugestão (cinza)</v>
+        <v>Sugeriu PROXIMIDADE REGIONAL — fallback de KM (âmbar)</v>
       </c>
       <c r="B6">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Missões com valor igual</v>
+        <v>Sugeriu MEMÓRIA DO AUDITOR — rota (roxo)</v>
       </c>
       <c r="B7">
-        <v>13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Missões com diferença</v>
+        <v>Sugeriu MEMÓRIA DO AUDITOR — região (roxo)</v>
       </c>
       <c r="B8">
-        <v>55</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>SEM sugestão (cinza)</v>
+      </c>
+      <c r="B9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Missões com valor igual</v>
+      </c>
+      <c r="B10">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Missões com diferença</v>
+      </c>
+      <c r="B11">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>Diferença total (R$)</v>
       </c>
-      <c r="B9" t="str">
-        <v>-159.955,32</v>
+      <c r="B12" t="str">
+        <v>-44.976,31</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -545,58 +569,58 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>GTM-5053</v>
+        <v>GTM-5090</v>
       </c>
       <c r="B2" t="str">
-        <v>Em Viagem</v>
+        <v>Cancelada</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-05-19T21:00:00+00:00</v>
+        <v>2026-05-20T17:27:00+00:00</v>
       </c>
       <c r="D2" t="str">
-        <v>AV. JÚLIA GAIOLI, 740 - ÁGUA CHATA, GUARULHOS - SP, 07251-500</v>
+        <v>FLORIANÓPOLIS, SC</v>
       </c>
       <c r="E2" t="str">
-        <v>R. NORMA DE ARAUJO BATISTA, 951 - DISTRITO INDUSTRIAL, JOÃO PESSOA - PB, 58088</v>
+        <v>FLORIANÓPOLIS, SC</v>
       </c>
       <c r="F2">
-        <v>2772.5</v>
+        <v>0</v>
       </c>
       <c r="G2" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H2">
-        <v>22635.93</v>
+        <v>8610.28</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2">
-        <v>22635.93</v>
+        <v>8610.28</v>
       </c>
       <c r="K2" t="str">
-        <v>(nenhuma)</v>
+        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
       </c>
       <c r="L2" t="str">
-        <v>none</v>
+        <v>region_band</v>
       </c>
       <c r="M2" t="str">
-        <v>SUDESTE</v>
+        <v>SUL</v>
       </c>
       <c r="N2">
-        <v>2800</v>
+        <v>100</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>690</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>690</v>
       </c>
       <c r="Q2">
-        <v>-22635.93</v>
+        <v>-7920.28</v>
       </c>
       <c r="R2" t="str">
-        <v>Sem tabela DHL para SUDESTE + 2800km — selecione manualmente</v>
+        <v>Sugestão por Proximidade (SUL + 100km)</v>
       </c>
       <c r="S2" t="str">
         <v/>
@@ -604,46 +628,46 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>GTM-5166</v>
+        <v>GTM-5020</v>
       </c>
       <c r="B3" t="str">
-        <v>Solicitada</v>
+        <v>Recusada</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-05-23T08:30:00+00:00</v>
+        <v>2026-05-19T01:30:00+00:00</v>
       </c>
       <c r="D3" t="str">
-        <v>Av. Júlia Gaioli, 740 - Água Chata, Guarulhos - SP, 07251-500</v>
+        <v>JANDIRA, SP</v>
       </c>
       <c r="E3" t="str">
-        <v>Estr. da Pedreira, 242 - PEDREIRA, Nova Santa Rita - RS, 92480-000</v>
+        <v>SÃO PAULO, SP</v>
       </c>
       <c r="F3">
-        <v>1178.1</v>
+        <v>37.9</v>
       </c>
       <c r="G3" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H3">
-        <v>12370.38</v>
+        <v>6513.6</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3">
-        <v>12370.38</v>
+        <v>6513.6</v>
       </c>
       <c r="K3" t="str">
-        <v>(nenhuma)</v>
+        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
       </c>
       <c r="L3" t="str">
-        <v>none</v>
+        <v>region_band</v>
       </c>
       <c r="M3" t="str">
         <v>SUDESTE</v>
       </c>
       <c r="N3">
-        <v>1200</v>
+        <v>100</v>
       </c>
       <c r="O3">
         <v>0</v>
@@ -652,10 +676,10 @@
         <v>0</v>
       </c>
       <c r="Q3">
-        <v>-12370.38</v>
+        <v>-6513.6</v>
       </c>
       <c r="R3" t="str">
-        <v>Sem tabela DHL para SUDESTE + 1200km — selecione manualmente</v>
+        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
       </c>
       <c r="S3" t="str">
         <v/>
@@ -663,22 +687,22 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>GTM-5159</v>
+        <v>GTM-5166</v>
       </c>
       <c r="B4" t="str">
-        <v>Em Viagem</v>
+        <v>Solicitada</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-05-22T15:50:00+00:00</v>
+        <v>2026-05-23T08:30:00+00:00</v>
       </c>
       <c r="D4" t="str">
-        <v>AV. JÚLIA GAIOLI, 740 - ÁGUA CHATA, GUARULHOS - SP, 07251-500</v>
+        <v>Av. Júlia Gaioli, 740 - Água Chata, Guarulhos - SP, 07251-500</v>
       </c>
       <c r="E4" t="str">
-        <v>AV. INDUSTRIAL BELGRAF, 865 - BAIRRO INDUSTRIAL, ELDORADO DO SUL - RS, 92990-000</v>
+        <v>Estr. da Pedreira, 242 - PEDREIRA, Nova Santa Rita - RS, 92480-000</v>
       </c>
       <c r="F4">
-        <v>1175.9</v>
+        <v>1178.1</v>
       </c>
       <c r="G4" t="str">
         <v>(não identificada)</v>
@@ -693,10 +717,10 @@
         <v>12370.38</v>
       </c>
       <c r="K4" t="str">
-        <v>(nenhuma)</v>
+        <v>REGIÃO - SUDESTE - BARUERI-NOVA SANTA RITA 1158KM</v>
       </c>
       <c r="L4" t="str">
-        <v>none</v>
+        <v>region_any_km</v>
       </c>
       <c r="M4" t="str">
         <v>SUDESTE</v>
@@ -705,16 +729,16 @@
         <v>1200</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>7990.2</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>7990.2</v>
       </c>
       <c r="Q4">
-        <v>-12370.38</v>
+        <v>-4380.18</v>
       </c>
       <c r="R4" t="str">
-        <v>Sem tabela DHL para SUDESTE + 1200km — selecione manualmente</v>
+        <v>Proximidade Regional (SUDESTE, mais próxima de 1178km)</v>
       </c>
       <c r="S4" t="str">
         <v/>
@@ -722,58 +746,58 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>GTM-5123</v>
+        <v>GTM-5159</v>
       </c>
       <c r="B5" t="str">
-        <v>Cancelada</v>
+        <v>Em Viagem</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-05-21T16:00:00+00:00</v>
+        <v>2026-05-22T15:50:00+00:00</v>
       </c>
       <c r="D5" t="str">
-        <v>VARGINHA, MG</v>
+        <v>AV. JÚLIA GAIOLI, 740 - ÁGUA CHATA, GUARULHOS - SP, 07251-500</v>
       </c>
       <c r="E5" t="str">
-        <v>SANTA ROSA, RS</v>
+        <v>AV. INDUSTRIAL BELGRAF, 865 - BAIRRO INDUSTRIAL, ELDORADO DO SUL - RS, 92990-000</v>
       </c>
       <c r="F5">
-        <v>1479.93</v>
+        <v>1175.9</v>
       </c>
       <c r="G5" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H5">
-        <v>11901.12</v>
+        <v>12370.38</v>
       </c>
       <c r="I5">
         <v>0</v>
       </c>
       <c r="J5">
-        <v>11901.12</v>
+        <v>12370.38</v>
       </c>
       <c r="K5" t="str">
-        <v>(nenhuma)</v>
+        <v>REGIÃO - SUDESTE - BARUERI-NOVA SANTA RITA 1158KM</v>
       </c>
       <c r="L5" t="str">
-        <v>none</v>
+        <v>region_any_km</v>
       </c>
       <c r="M5" t="str">
         <v>SUDESTE</v>
       </c>
       <c r="N5">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>7990.2</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>7990.2</v>
       </c>
       <c r="Q5">
-        <v>-11901.12</v>
+        <v>-4380.18</v>
       </c>
       <c r="R5" t="str">
-        <v>Sem tabela DHL para SUDESTE + 1500km — selecione manualmente</v>
+        <v>Proximidade Regional (SUDESTE, mais próxima de 1176km)</v>
       </c>
       <c r="S5" t="str">
         <v/>
@@ -781,58 +805,58 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>GTM-5069</v>
+        <v>GTM-5053</v>
       </c>
       <c r="B6" t="str">
-        <v>Concluída</v>
+        <v>Em Viagem</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-05-20T08:00:00+00:00</v>
+        <v>2026-05-19T21:00:00+00:00</v>
       </c>
       <c r="D6" t="str">
-        <v>ROD. HÉLIO SMIDT, S/N - SETOR 3 - TERMINAL COURIER, GUARULHOS - SP, 07190-100</v>
+        <v>AV. JÚLIA GAIOLI, 740 - ÁGUA CHATA, GUARULHOS - SP, 07251-500</v>
       </c>
       <c r="E6" t="str">
-        <v>SERRA, ES</v>
+        <v>R. NORMA DE ARAUJO BATISTA, 951 - DISTRITO INDUSTRIAL, JOÃO PESSOA - PB, 58088</v>
       </c>
       <c r="F6">
-        <v>945.9</v>
+        <v>2772.5</v>
       </c>
       <c r="G6" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H6">
-        <v>9920.95</v>
+        <v>22635.93</v>
       </c>
       <c r="I6">
-        <v>177.5</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <v>10098.45</v>
+        <v>22635.93</v>
       </c>
       <c r="K6" t="str">
-        <v>(nenhuma)</v>
+        <v>REGIÃO - SUDESTE - EXTREMA-CABEDELO 2650KM</v>
       </c>
       <c r="L6" t="str">
-        <v>none</v>
+        <v>region_any_km</v>
       </c>
       <c r="M6" t="str">
         <v>SUDESTE</v>
       </c>
       <c r="N6">
-        <v>900</v>
+        <v>2800</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>26558.75</v>
       </c>
       <c r="P6">
-        <v>177.5</v>
+        <v>26558.75</v>
       </c>
       <c r="Q6">
-        <v>-9920.95</v>
+        <v>3922.82</v>
       </c>
       <c r="R6" t="str">
-        <v>Sem tabela DHL para SUDESTE + 900km — selecione manualmente</v>
+        <v>Proximidade Regional (SUDESTE, mais próxima de 2773km)</v>
       </c>
       <c r="S6" t="str">
         <v/>
@@ -840,34 +864,34 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>GTM-5070</v>
+        <v>GTM-5139</v>
       </c>
       <c r="B7" t="str">
         <v>Concluída</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-05-20T10:00:00+00:00</v>
+        <v>2026-05-22T00:25:00+00:00</v>
       </c>
       <c r="D7" t="str">
-        <v>ROD. HÉLIO SMIDT, S/N - SETOR 3 - TERMINAL COURIER, GUARULHOS - SP, 07190-100</v>
+        <v>ROD. FERNÃO DIAS</v>
       </c>
       <c r="E7" t="str">
-        <v>SERRA, ES</v>
+        <v>RAIO 400 KM — DESTINO A DEFINIR</v>
       </c>
       <c r="F7">
-        <v>945.9</v>
+        <v>400</v>
       </c>
       <c r="G7" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H7">
-        <v>9628.53</v>
+        <v>2760</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7">
-        <v>9628.53</v>
+        <v>2760</v>
       </c>
       <c r="K7" t="str">
         <v>(nenhuma)</v>
@@ -876,10 +900,10 @@
         <v>none</v>
       </c>
       <c r="M7" t="str">
-        <v>SUDESTE</v>
+        <v/>
       </c>
       <c r="N7">
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="O7">
         <v>0</v>
@@ -888,10 +912,10 @@
         <v>0</v>
       </c>
       <c r="Q7">
-        <v>-9628.53</v>
+        <v>-2760</v>
       </c>
       <c r="R7" t="str">
-        <v>Sem tabela DHL para SUDESTE + 900km — selecione manualmente</v>
+        <v>Origem sem UF identificada (faixa 400km) — selecione manualmente</v>
       </c>
       <c r="S7" t="str">
         <v/>
@@ -899,58 +923,58 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>GTM-5150</v>
+        <v>GTM-5097</v>
       </c>
       <c r="B8" t="str">
-        <v>Em Viagem</v>
+        <v>Concluída</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-05-22T04:00:00+00:00</v>
+        <v>2026-05-21T07:00:00+00:00</v>
       </c>
       <c r="D8" t="str">
-        <v>ESTR. DOS ALPES, 320 - JARDIM ITAQUITI, BARUERI - SP, 06423-080</v>
+        <v>AV. JÚLIA GAIOLI, 740 - ÁGUA CHATA, GUARULHOS - SP, 07251-500</v>
       </c>
       <c r="E8" t="str">
-        <v>BRASÍLIA - PLANO PILOTO, BRASÍLIA - DF</v>
+        <v>AV. TALMA RODRIGUES RIBEIRO, 147 - VILA NOVA DE COLARES, SERRA - ES, 29172-038</v>
       </c>
       <c r="F8">
-        <v>1012.7</v>
+        <v>935.1</v>
       </c>
       <c r="G8" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H8">
-        <v>7990.2</v>
+        <v>7412.45</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8">
-        <v>7990.2</v>
+        <v>7412.45</v>
       </c>
       <c r="K8" t="str">
-        <v>(nenhuma)</v>
+        <v>REGIÃO - SUDESTE - LOUVEIRA-APARECIDA DE GOIANIA 946KM</v>
       </c>
       <c r="L8" t="str">
-        <v>none</v>
+        <v>region_any_km</v>
       </c>
       <c r="M8" t="str">
         <v>SUDESTE</v>
       </c>
       <c r="N8">
-        <v>1000</v>
+        <v>900</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>9913.15</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>9913.15</v>
       </c>
       <c r="Q8">
-        <v>-7990.2</v>
+        <v>2500.7</v>
       </c>
       <c r="R8" t="str">
-        <v>Sem tabela DHL para SUDESTE + 1000km — selecione manualmente</v>
+        <v>Proximidade Regional (SUDESTE, mais próxima de 935km)</v>
       </c>
       <c r="S8" t="str">
         <v/>
@@ -958,58 +982,58 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>GTM-5090</v>
+        <v>GTM-5068</v>
       </c>
       <c r="B9" t="str">
-        <v>Cancelada</v>
+        <v>Concluída</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-05-20T17:27:00+00:00</v>
+        <v>2026-05-20T04:00:00+00:00</v>
       </c>
       <c r="D9" t="str">
-        <v>FLORIANÓPOLIS, SC</v>
+        <v>ROD. HÉLIO SMIDT, S/N - SETOR 3 - TERMINAL COURIER, GUARULHOS - SP, 07190-100</v>
       </c>
       <c r="E9" t="str">
-        <v>FLORIANÓPOLIS, SC</v>
+        <v>SERRA, ES</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>945.9</v>
       </c>
       <c r="G9" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H9">
-        <v>8610.28</v>
+        <v>7412.45</v>
       </c>
       <c r="I9">
         <v>0</v>
       </c>
       <c r="J9">
-        <v>8610.28</v>
+        <v>7412.45</v>
       </c>
       <c r="K9" t="str">
-        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
+        <v>REGIÃO - SUDESTE - LOUVEIRA-APARECIDA DE GOIANIA 946KM</v>
       </c>
       <c r="L9" t="str">
-        <v>region_band</v>
+        <v>region_any_km</v>
       </c>
       <c r="M9" t="str">
-        <v>SUL</v>
+        <v>SUDESTE</v>
       </c>
       <c r="N9">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="O9">
-        <v>690</v>
+        <v>9913.15</v>
       </c>
       <c r="P9">
-        <v>690</v>
+        <v>9913.15</v>
       </c>
       <c r="Q9">
-        <v>-7920.28</v>
+        <v>2500.7</v>
       </c>
       <c r="R9" t="str">
-        <v>Sugestão por Proximidade (SUL + 100km)</v>
+        <v>Proximidade Regional (SUDESTE, mais próxima de 946km)</v>
       </c>
       <c r="S9" t="str">
         <v/>
@@ -1017,46 +1041,46 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>GTM-5097</v>
+        <v>GTM-5129</v>
       </c>
       <c r="B10" t="str">
-        <v>Concluída</v>
+        <v>Recusada</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-05-21T07:00:00+00:00</v>
+        <v>2026-05-21T17:20:00+00:00</v>
       </c>
       <c r="D10" t="str">
-        <v>AV. JÚLIA GAIOLI, 740 - ÁGUA CHATA, GUARULHOS - SP, 07251-500</v>
+        <v>AV. ROCHA POMBO - SÃO CRISTÓVÃO, SÃO JOSÉ DOS PINHAIS - PR</v>
       </c>
       <c r="E10" t="str">
-        <v>AV. TALMA RODRIGUES RIBEIRO, 147 - VILA NOVA DE COLARES, SERRA - ES, 29172-038</v>
+        <v>R. FRANCISCO MUNÕZ MADRID, 625 - ROSEIRA DE SÃO SEBASTIÃO, SÃO JOSÉ DOS PINHAIS - PR, 83070-010</v>
       </c>
       <c r="F10">
-        <v>935.1</v>
+        <v>9.1</v>
       </c>
       <c r="G10" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H10">
-        <v>7412.45</v>
+        <v>2264.58</v>
       </c>
       <c r="I10">
         <v>0</v>
       </c>
       <c r="J10">
-        <v>7412.45</v>
+        <v>2264.58</v>
       </c>
       <c r="K10" t="str">
-        <v>(nenhuma)</v>
+        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
       </c>
       <c r="L10" t="str">
-        <v>none</v>
+        <v>region_band</v>
       </c>
       <c r="M10" t="str">
-        <v>SUDESTE</v>
+        <v>SUL</v>
       </c>
       <c r="N10">
-        <v>900</v>
+        <v>100</v>
       </c>
       <c r="O10">
         <v>0</v>
@@ -1065,10 +1089,10 @@
         <v>0</v>
       </c>
       <c r="Q10">
-        <v>-7412.45</v>
+        <v>-2264.58</v>
       </c>
       <c r="R10" t="str">
-        <v>Sem tabela DHL para SUDESTE + 900km — selecione manualmente</v>
+        <v>Sugestão por Proximidade (SUL + 100km)</v>
       </c>
       <c r="S10" t="str">
         <v/>
@@ -1076,34 +1100,34 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>GTM-5068</v>
+        <v>GTM-5076</v>
       </c>
       <c r="B11" t="str">
         <v>Concluída</v>
       </c>
       <c r="C11" t="str">
-        <v>2026-05-20T04:00:00+00:00</v>
+        <v>2026-05-20T11:00:00+00:00</v>
       </c>
       <c r="D11" t="str">
-        <v>ROD. HÉLIO SMIDT, S/N - SETOR 3 - TERMINAL COURIER, GUARULHOS - SP, 07190-100</v>
+        <v>LAGO SUL, BRASÍLIA - DF, 71608-900</v>
       </c>
       <c r="E11" t="str">
-        <v>SERRA, ES</v>
+        <v>BRASÍLIA - DF</v>
       </c>
       <c r="F11">
-        <v>945.9</v>
+        <v>13.1</v>
       </c>
       <c r="G11" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H11">
-        <v>7412.45</v>
+        <v>2264.58</v>
       </c>
       <c r="I11">
         <v>0</v>
       </c>
       <c r="J11">
-        <v>7412.45</v>
+        <v>2264.58</v>
       </c>
       <c r="K11" t="str">
         <v>(nenhuma)</v>
@@ -1112,10 +1136,10 @@
         <v>none</v>
       </c>
       <c r="M11" t="str">
-        <v>SUDESTE</v>
+        <v>CENTRO-OESTE</v>
       </c>
       <c r="N11">
-        <v>900</v>
+        <v>100</v>
       </c>
       <c r="O11">
         <v>0</v>
@@ -1124,10 +1148,10 @@
         <v>0</v>
       </c>
       <c r="Q11">
-        <v>-7412.45</v>
+        <v>-2264.58</v>
       </c>
       <c r="R11" t="str">
-        <v>Sem tabela DHL para SUDESTE + 900km — selecione manualmente</v>
+        <v>Sem tabela DHL para CENTRO-OESTE — selecione manualmente</v>
       </c>
       <c r="S11" t="str">
         <v/>
@@ -1135,43 +1159,43 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>GTM-5020</v>
+        <v>GTM-5038</v>
       </c>
       <c r="B12" t="str">
-        <v>Recusada</v>
+        <v>Concluída</v>
       </c>
       <c r="C12" t="str">
-        <v>2026-05-19T01:30:00+00:00</v>
+        <v>2026-05-19T09:30:00+00:00</v>
       </c>
       <c r="D12" t="str">
-        <v>JANDIRA, SP</v>
+        <v>R. TODICA, 2-346 - SÍTIO DE RECREIO IPÊ, GOIÂNIA - GO, 74594-111</v>
       </c>
       <c r="E12" t="str">
-        <v>SÃO PAULO, SP</v>
+        <v>R. PORTO NACIONAL, 265 - JARDIM GUANABARA, GOIÂNIA - GO, 74675-690</v>
       </c>
       <c r="F12">
-        <v>37.9</v>
+        <v>5.1</v>
       </c>
       <c r="G12" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H12">
-        <v>6513.6</v>
+        <v>2264.58</v>
       </c>
       <c r="I12">
         <v>0</v>
       </c>
       <c r="J12">
-        <v>6513.6</v>
+        <v>2264.58</v>
       </c>
       <c r="K12" t="str">
-        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
+        <v>(nenhuma)</v>
       </c>
       <c r="L12" t="str">
-        <v>region_band</v>
+        <v>none</v>
       </c>
       <c r="M12" t="str">
-        <v>SUDESTE</v>
+        <v>CENTRO-OESTE</v>
       </c>
       <c r="N12">
         <v>100</v>
@@ -1183,10 +1207,10 @@
         <v>0</v>
       </c>
       <c r="Q12">
-        <v>-6513.6</v>
+        <v>-2264.58</v>
       </c>
       <c r="R12" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
+        <v>Sem tabela DHL para CENTRO-OESTE — selecione manualmente</v>
       </c>
       <c r="S12" t="str">
         <v/>
@@ -1194,34 +1218,34 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>GTM-5135</v>
+        <v>GTM-5149</v>
       </c>
       <c r="B13" t="str">
         <v>Concluída</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-05-21T21:40:00+00:00</v>
+        <v>2026-05-22T01:10:00+00:00</v>
       </c>
       <c r="D13" t="str">
-        <v>R. VER. GERMANO LUÍS VIÊIRA - ITAIPAVA, ITAJAÍ - SC</v>
+        <v>AV. NORBERTO JOSÉ TEIXEIRA - APARECIDA DE GOIÂNIA, GO</v>
       </c>
       <c r="E13" t="str">
-        <v>AV. CECI - TAMBORÉ, BARUERI - SP, 06460-120</v>
+        <v>RAIO 200 KM — DESTINO A DEFINIR</v>
       </c>
       <c r="F13">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="G13" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H13">
-        <v>3989.17</v>
+        <v>2070</v>
       </c>
       <c r="I13">
         <v>0</v>
       </c>
       <c r="J13">
-        <v>3989.17</v>
+        <v>2070</v>
       </c>
       <c r="K13" t="str">
         <v>(nenhuma)</v>
@@ -1230,10 +1254,10 @@
         <v>none</v>
       </c>
       <c r="M13" t="str">
-        <v>SUL</v>
+        <v>CENTRO-OESTE</v>
       </c>
       <c r="N13">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="O13">
         <v>0</v>
@@ -1242,10 +1266,10 @@
         <v>0</v>
       </c>
       <c r="Q13">
-        <v>-3989.17</v>
+        <v>-2070</v>
       </c>
       <c r="R13" t="str">
-        <v>Sem tabela DHL para SUL + 600km — selecione manualmente</v>
+        <v>Sem tabela DHL para CENTRO-OESTE — selecione manualmente</v>
       </c>
       <c r="S13" t="str">
         <v/>
@@ -1253,58 +1277,58 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>GTM-5134</v>
+        <v>GTM-5156</v>
       </c>
       <c r="B14" t="str">
         <v>Concluída</v>
       </c>
       <c r="C14" t="str">
-        <v>2026-05-21T21:40:00+00:00</v>
+        <v>2026-05-22T10:00:00+00:00</v>
       </c>
       <c r="D14" t="str">
-        <v>R. VER. GERMANO LUÍS VIÊIRA - ITAIPAVA, ITAJAÍ - SC</v>
+        <v>SAPUCAIA DO SUL, RS</v>
       </c>
       <c r="E14" t="str">
-        <v>AV. CECI - TAMBORÉ, BARUERI - SP, 06460-120</v>
+        <v>PORTAL DA SERRA, DOIS IRMÃOS - RS, 93950-000</v>
       </c>
       <c r="F14">
-        <v>600</v>
+        <v>33.5</v>
       </c>
       <c r="G14" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H14">
-        <v>3675</v>
+        <v>2264.58</v>
       </c>
       <c r="I14">
         <v>0</v>
       </c>
       <c r="J14">
-        <v>3675</v>
+        <v>2264.58</v>
       </c>
       <c r="K14" t="str">
-        <v>(nenhuma)</v>
+        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
       </c>
       <c r="L14" t="str">
-        <v>none</v>
+        <v>region_band</v>
       </c>
       <c r="M14" t="str">
         <v>SUL</v>
       </c>
       <c r="N14">
-        <v>600</v>
+        <v>100</v>
       </c>
       <c r="O14">
-        <v>0</v>
+        <v>690</v>
       </c>
       <c r="P14">
-        <v>0</v>
+        <v>690</v>
       </c>
       <c r="Q14">
-        <v>-3675</v>
+        <v>-1574.58</v>
       </c>
       <c r="R14" t="str">
-        <v>Sem tabela DHL para SUL + 600km — selecione manualmente</v>
+        <v>Sugestão por Proximidade (SUL + 100km)</v>
       </c>
       <c r="S14" t="str">
         <v/>
@@ -1312,58 +1336,58 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>GTM-5051</v>
+        <v>GTM-5115</v>
       </c>
       <c r="B15" t="str">
         <v>Concluída</v>
       </c>
       <c r="C15" t="str">
-        <v>2026-05-19T20:30:00+00:00</v>
+        <v>2026-05-21T12:00:00+00:00</v>
       </c>
       <c r="D15" t="str">
-        <v>R. VER. GERMANO LUÍS VIÊIRA, 1-1300 - ITAIPAVA, ITAJAÍ - SC, 88316-701</v>
+        <v>AV. ROZA HELENA SCHORLING ALBUQUERQUE, S/N - AEROPORTO, VITÓRIA - ES, 29075-685</v>
       </c>
       <c r="E15" t="str">
-        <v>AV. CECI, 1900 - JARDIM MUTINGA, BARUERI - SP, 06460-120</v>
+        <v>CARIACICA, ES, 29156-113</v>
       </c>
       <c r="F15">
-        <v>600.9</v>
+        <v>29.4</v>
       </c>
       <c r="G15" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H15">
-        <v>3675</v>
+        <v>2264.58</v>
       </c>
       <c r="I15">
-        <v>53.7</v>
+        <v>0</v>
       </c>
       <c r="J15">
-        <v>3728.7</v>
+        <v>2264.58</v>
       </c>
       <c r="K15" t="str">
-        <v>(nenhuma)</v>
+        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
       </c>
       <c r="L15" t="str">
-        <v>none</v>
+        <v>region_band</v>
       </c>
       <c r="M15" t="str">
-        <v>SUL</v>
+        <v>SUDESTE</v>
       </c>
       <c r="N15">
-        <v>600</v>
+        <v>100</v>
       </c>
       <c r="O15">
-        <v>0</v>
+        <v>690</v>
       </c>
       <c r="P15">
-        <v>53.7</v>
+        <v>690</v>
       </c>
       <c r="Q15">
-        <v>-3675</v>
+        <v>-1574.58</v>
       </c>
       <c r="R15" t="str">
-        <v>Sem tabela DHL para SUL + 600km — selecione manualmente</v>
+        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
       </c>
       <c r="S15" t="str">
         <v/>
@@ -1371,58 +1395,58 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>GTM-5139</v>
+        <v>GTM-5104</v>
       </c>
       <c r="B16" t="str">
         <v>Concluída</v>
       </c>
       <c r="C16" t="str">
-        <v>2026-05-22T00:25:00+00:00</v>
+        <v>2026-05-21T10:30:00+00:00</v>
       </c>
       <c r="D16" t="str">
-        <v>ROD. FERNÃO DIAS</v>
+        <v>AV. DEP. DIOMÍCIO FREITAS, 3125 - CARIANOS, FLORIANÓPOLIS - SC, 88047-402</v>
       </c>
       <c r="E16" t="str">
-        <v>RAIO 400 KM — DESTINO A DEFINIR</v>
+        <v>SC-407, 2800 - VENDAVAL, BIGUAÇU - SC, 88164-169</v>
       </c>
       <c r="F16">
-        <v>400</v>
+        <v>33.6</v>
       </c>
       <c r="G16" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H16">
-        <v>2760</v>
+        <v>2264.58</v>
       </c>
       <c r="I16">
         <v>0</v>
       </c>
       <c r="J16">
-        <v>2760</v>
+        <v>2264.58</v>
       </c>
       <c r="K16" t="str">
-        <v>(nenhuma)</v>
+        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
       </c>
       <c r="L16" t="str">
-        <v>none</v>
+        <v>region_band</v>
       </c>
       <c r="M16" t="str">
-        <v/>
+        <v>SUL</v>
       </c>
       <c r="N16">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="O16">
-        <v>0</v>
+        <v>690</v>
       </c>
       <c r="P16">
-        <v>0</v>
+        <v>690</v>
       </c>
       <c r="Q16">
-        <v>-2760</v>
+        <v>-1574.58</v>
       </c>
       <c r="R16" t="str">
-        <v>Origem sem UF identificada (faixa 400km) — selecione manualmente</v>
+        <v>Sugestão por Proximidade (SUL + 100km)</v>
       </c>
       <c r="S16" t="str">
         <v/>
@@ -1430,22 +1454,22 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>GTM-5129</v>
+        <v>GTM-5037</v>
       </c>
       <c r="B17" t="str">
-        <v>Recusada</v>
+        <v>Concluída</v>
       </c>
       <c r="C17" t="str">
-        <v>2026-05-21T17:20:00+00:00</v>
+        <v>2026-05-19T12:00:00+00:00</v>
       </c>
       <c r="D17" t="str">
-        <v>AV. ROCHA POMBO - SÃO CRISTÓVÃO, SÃO JOSÉ DOS PINHAIS - PR</v>
+        <v>RIO DE JANEIRO, RJ</v>
       </c>
       <c r="E17" t="str">
-        <v>R. FRANCISCO MUNÕZ MADRID, 625 - ROSEIRA DE SÃO SEBASTIÃO, SÃO JOSÉ DOS PINHAIS - PR, 83070-010</v>
+        <v>RIO DE JANEIRO, RJ</v>
       </c>
       <c r="F17">
-        <v>9.1</v>
+        <v>0</v>
       </c>
       <c r="G17" t="str">
         <v>(não identificada)</v>
@@ -1460,28 +1484,28 @@
         <v>2264.58</v>
       </c>
       <c r="K17" t="str">
-        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
+        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
       </c>
       <c r="L17" t="str">
         <v>region_band</v>
       </c>
       <c r="M17" t="str">
-        <v>SUL</v>
+        <v>SUDESTE</v>
       </c>
       <c r="N17">
         <v>100</v>
       </c>
       <c r="O17">
-        <v>0</v>
+        <v>690</v>
       </c>
       <c r="P17">
-        <v>0</v>
+        <v>690</v>
       </c>
       <c r="Q17">
-        <v>-2264.58</v>
+        <v>-1574.58</v>
       </c>
       <c r="R17" t="str">
-        <v>Sugestão por Proximidade (SUL + 100km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
       </c>
       <c r="S17" t="str">
         <v/>
@@ -1489,22 +1513,22 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>GTM-5076</v>
+        <v>GTM-5085</v>
       </c>
       <c r="B18" t="str">
         <v>Concluída</v>
       </c>
       <c r="C18" t="str">
-        <v>2026-05-20T11:00:00+00:00</v>
+        <v>2026-05-20T18:43:00+00:00</v>
       </c>
       <c r="D18" t="str">
-        <v>LAGO SUL, BRASÍLIA - DF, 71608-900</v>
+        <v>ROD. CEL. PM NELSON TRANCHESI, 1730 - ITAQUI, ITAPEVI - SP, 06696-110</v>
       </c>
       <c r="E18" t="str">
-        <v>BRASÍLIA - DF</v>
+        <v>ESTR. DOS ALPES, 320 - JARDIM ITAQUITI, BARUERI - SP, 06423-080</v>
       </c>
       <c r="F18">
-        <v>13.1</v>
+        <v>8.1</v>
       </c>
       <c r="G18" t="str">
         <v>(não identificada)</v>
@@ -1513,34 +1537,34 @@
         <v>2264.58</v>
       </c>
       <c r="I18">
-        <v>0</v>
+        <v>5.4</v>
       </c>
       <c r="J18">
-        <v>2264.58</v>
+        <v>2269.98</v>
       </c>
       <c r="K18" t="str">
-        <v>(nenhuma)</v>
+        <v>REGIÃO - SUDESTE - ITAPEVI-BARUERI 100KM</v>
       </c>
       <c r="L18" t="str">
-        <v>none</v>
+        <v>exact_route</v>
       </c>
       <c r="M18" t="str">
-        <v>CENTRO-OESTE</v>
+        <v>SUDESTE</v>
       </c>
       <c r="N18">
         <v>100</v>
       </c>
       <c r="O18">
-        <v>0</v>
+        <v>695.4</v>
       </c>
       <c r="P18">
-        <v>0</v>
+        <v>700.8</v>
       </c>
       <c r="Q18">
-        <v>-2264.58</v>
+        <v>-1569.18</v>
       </c>
       <c r="R18" t="str">
-        <v>Sem tabela DHL para CENTRO-OESTE + 100km — selecione manualmente</v>
+        <v>Rota Exata (SUDESTE + 100km)</v>
       </c>
       <c r="S18" t="str">
         <v/>
@@ -1548,22 +1572,22 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>GTM-5038</v>
+        <v>GTM-5071</v>
       </c>
       <c r="B19" t="str">
         <v>Concluída</v>
       </c>
       <c r="C19" t="str">
-        <v>2026-05-19T09:30:00+00:00</v>
+        <v>2026-05-20T10:30:00+00:00</v>
       </c>
       <c r="D19" t="str">
-        <v>R. TODICA, 2-346 - SÍTIO DE RECREIO IPÊ, GOIÂNIA - GO, 74594-111</v>
+        <v>FLORIANÓPOLIS, SC</v>
       </c>
       <c r="E19" t="str">
-        <v>R. PORTO NACIONAL, 265 - JARDIM GUANABARA, GOIÂNIA - GO, 74675-690</v>
+        <v>FLORIANÓPOLIS, SC</v>
       </c>
       <c r="F19">
-        <v>5.1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="str">
         <v>(não identificada)</v>
@@ -1578,28 +1602,28 @@
         <v>2264.58</v>
       </c>
       <c r="K19" t="str">
-        <v>(nenhuma)</v>
+        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
       </c>
       <c r="L19" t="str">
-        <v>none</v>
+        <v>region_band</v>
       </c>
       <c r="M19" t="str">
-        <v>CENTRO-OESTE</v>
+        <v>SUL</v>
       </c>
       <c r="N19">
         <v>100</v>
       </c>
       <c r="O19">
-        <v>0</v>
+        <v>702.08</v>
       </c>
       <c r="P19">
-        <v>0</v>
+        <v>702.08</v>
       </c>
       <c r="Q19">
-        <v>-2264.58</v>
+        <v>-1562.5</v>
       </c>
       <c r="R19" t="str">
-        <v>Sem tabela DHL para CENTRO-OESTE + 100km — selecione manualmente</v>
+        <v>Sugestão por Proximidade (SUL + 100km)</v>
       </c>
       <c r="S19" t="str">
         <v/>
@@ -1607,58 +1631,58 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>GTM-5149</v>
+        <v>GTM-5019</v>
       </c>
       <c r="B20" t="str">
         <v>Concluída</v>
       </c>
       <c r="C20" t="str">
-        <v>2026-05-22T01:10:00+00:00</v>
+        <v>2026-05-19T10:30:00+00:00</v>
       </c>
       <c r="D20" t="str">
-        <v>AV. NORBERTO JOSÉ TEIXEIRA - APARECIDA DE GOIÂNIA, GO</v>
+        <v>FLORIANÓPOLIS, SC</v>
       </c>
       <c r="E20" t="str">
-        <v>RAIO 200 KM — DESTINO A DEFINIR</v>
+        <v>FLORIANÓPOLIS, SC</v>
       </c>
       <c r="F20">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="G20" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H20">
-        <v>2070</v>
+        <v>2264.58</v>
       </c>
       <c r="I20">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="J20">
-        <v>2070</v>
+        <v>2299.58</v>
       </c>
       <c r="K20" t="str">
-        <v>(nenhuma)</v>
+        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
       </c>
       <c r="L20" t="str">
-        <v>none</v>
+        <v>region_band</v>
       </c>
       <c r="M20" t="str">
-        <v>CENTRO-OESTE</v>
+        <v>SUL</v>
       </c>
       <c r="N20">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="O20">
-        <v>0</v>
+        <v>725</v>
       </c>
       <c r="P20">
-        <v>0</v>
+        <v>760</v>
       </c>
       <c r="Q20">
-        <v>-2070</v>
+        <v>-1539.58</v>
       </c>
       <c r="R20" t="str">
-        <v>Sem tabela DHL para CENTRO-OESTE + 200km — selecione manualmente</v>
+        <v>Sugestão por Proximidade (SUL + 100km)</v>
       </c>
       <c r="S20" t="str">
         <v/>
@@ -1666,22 +1690,22 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>GTM-5156</v>
+        <v>GTM-5160</v>
       </c>
       <c r="B21" t="str">
-        <v>Concluída</v>
+        <v>Em Viagem</v>
       </c>
       <c r="C21" t="str">
-        <v>2026-05-22T10:00:00+00:00</v>
+        <v>2026-05-22T16:30:00+00:00</v>
       </c>
       <c r="D21" t="str">
-        <v>SAPUCAIA DO SUL, RS</v>
+        <v>AV. SEVERO DULLIUS, 90010 - ANCHIETA, PORTO ALEGRE - RS, 90200-310</v>
       </c>
       <c r="E21" t="str">
-        <v>PORTAL DA SERRA, DOIS IRMÃOS - RS, 93950-000</v>
+        <v>AV. BORGES DE MEDEIROS, 1771 - COLONIAL, SAPUCAIA DO SUL - RS, 93212-110</v>
       </c>
       <c r="F21">
-        <v>33.5</v>
+        <v>22.7</v>
       </c>
       <c r="G21" t="str">
         <v>(não identificada)</v>
@@ -1708,13 +1732,13 @@
         <v>100</v>
       </c>
       <c r="O21">
-        <v>690</v>
+        <v>726.25</v>
       </c>
       <c r="P21">
-        <v>690</v>
+        <v>726.25</v>
       </c>
       <c r="Q21">
-        <v>-1574.58</v>
+        <v>-1538.33</v>
       </c>
       <c r="R21" t="str">
         <v>Sugestão por Proximidade (SUL + 100km)</v>
@@ -1725,22 +1749,22 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>GTM-5115</v>
+        <v>GTM-5161</v>
       </c>
       <c r="B22" t="str">
-        <v>Concluída</v>
+        <v>Em Viagem</v>
       </c>
       <c r="C22" t="str">
-        <v>2026-05-21T12:00:00+00:00</v>
+        <v>2026-05-22T16:30:00+00:00</v>
       </c>
       <c r="D22" t="str">
-        <v>AV. ROZA HELENA SCHORLING ALBUQUERQUE, S/N - AEROPORTO, VITÓRIA - ES, 29075-685</v>
+        <v>AV. SEVERO DULLIUS, 90010 - ANCHIETA, PORTO ALEGRE - RS, 90200-310</v>
       </c>
       <c r="E22" t="str">
-        <v>CARIACICA, ES, 29156-113</v>
+        <v>AV. BORGES DE MEDEIROS, 1771 - COLONIAL, SAPUCAIA DO SUL - RS, 93212-110</v>
       </c>
       <c r="F22">
-        <v>29.4</v>
+        <v>22.7</v>
       </c>
       <c r="G22" t="str">
         <v>(não identificada)</v>
@@ -1755,28 +1779,28 @@
         <v>2264.58</v>
       </c>
       <c r="K22" t="str">
-        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
+        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
       </c>
       <c r="L22" t="str">
         <v>region_band</v>
       </c>
       <c r="M22" t="str">
-        <v>SUDESTE</v>
+        <v>SUL</v>
       </c>
       <c r="N22">
         <v>100</v>
       </c>
       <c r="O22">
-        <v>690</v>
+        <v>726.25</v>
       </c>
       <c r="P22">
-        <v>690</v>
+        <v>726.25</v>
       </c>
       <c r="Q22">
-        <v>-1574.58</v>
+        <v>-1538.33</v>
       </c>
       <c r="R22" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
+        <v>Sugestão por Proximidade (SUL + 100km)</v>
       </c>
       <c r="S22" t="str">
         <v/>
@@ -1784,22 +1808,22 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>GTM-5104</v>
+        <v>GTM-5036</v>
       </c>
       <c r="B23" t="str">
         <v>Concluída</v>
       </c>
       <c r="C23" t="str">
-        <v>2026-05-21T10:30:00+00:00</v>
+        <v>2026-05-19T10:00:00+00:00</v>
       </c>
       <c r="D23" t="str">
-        <v>AV. DEP. DIOMÍCIO FREITAS, 3125 - CARIANOS, FLORIANÓPOLIS - SC, 88047-402</v>
+        <v>RIO DE JANEIRO, RJ</v>
       </c>
       <c r="E23" t="str">
-        <v>SC-407, 2800 - VENDAVAL, BIGUAÇU - SC, 88164-169</v>
+        <v>RIO DE JANEIRO, RJ</v>
       </c>
       <c r="F23">
-        <v>33.6</v>
+        <v>0</v>
       </c>
       <c r="G23" t="str">
         <v>(não identificada)</v>
@@ -1814,28 +1838,28 @@
         <v>2264.58</v>
       </c>
       <c r="K23" t="str">
-        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
+        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
       </c>
       <c r="L23" t="str">
         <v>region_band</v>
       </c>
       <c r="M23" t="str">
-        <v>SUL</v>
+        <v>SUDESTE</v>
       </c>
       <c r="N23">
         <v>100</v>
       </c>
       <c r="O23">
-        <v>690</v>
+        <v>743.17</v>
       </c>
       <c r="P23">
-        <v>690</v>
+        <v>743.17</v>
       </c>
       <c r="Q23">
-        <v>-1574.58</v>
+        <v>-1521.41</v>
       </c>
       <c r="R23" t="str">
-        <v>Sugestão por Proximidade (SUL + 100km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
       </c>
       <c r="S23" t="str">
         <v/>
@@ -1843,22 +1867,22 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>GTM-5037</v>
+        <v>GTM-5030</v>
       </c>
       <c r="B24" t="str">
         <v>Concluída</v>
       </c>
       <c r="C24" t="str">
-        <v>2026-05-19T12:00:00+00:00</v>
+        <v>2026-05-19T09:30:00+00:00</v>
       </c>
       <c r="D24" t="str">
-        <v>RIO DE JANEIRO, RJ</v>
+        <v>R. 20 DE AGOSTO, 1204 - COLONIAL, SAPUCAIA DO SUL - RS, 93212-710</v>
       </c>
       <c r="E24" t="str">
-        <v>RIO DE JANEIRO, RJ</v>
+        <v>BR-116, 7350 - PORTAL DA SERRA, DOIS IRMÃOS - RS, 93950-000</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>31.7</v>
       </c>
       <c r="G24" t="str">
         <v>(não identificada)</v>
@@ -1867,34 +1891,34 @@
         <v>2264.58</v>
       </c>
       <c r="I24">
-        <v>0</v>
+        <v>5.85</v>
       </c>
       <c r="J24">
-        <v>2264.58</v>
+        <v>2270.43</v>
       </c>
       <c r="K24" t="str">
-        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
+        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
       </c>
       <c r="L24" t="str">
         <v>region_band</v>
       </c>
       <c r="M24" t="str">
-        <v>SUDESTE</v>
+        <v>SUL</v>
       </c>
       <c r="N24">
         <v>100</v>
       </c>
       <c r="O24">
-        <v>690</v>
+        <v>778.02</v>
       </c>
       <c r="P24">
-        <v>690</v>
+        <v>783.87</v>
       </c>
       <c r="Q24">
-        <v>-1574.58</v>
+        <v>-1486.56</v>
       </c>
       <c r="R24" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
+        <v>Sugestão por Proximidade (SUL + 100km)</v>
       </c>
       <c r="S24" t="str">
         <v/>
@@ -1902,22 +1926,22 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>GTM-5085</v>
+        <v>GTM-5155</v>
       </c>
       <c r="B25" t="str">
         <v>Concluída</v>
       </c>
       <c r="C25" t="str">
-        <v>2026-05-20T18:43:00+00:00</v>
+        <v>2026-05-22T09:00:00+00:00</v>
       </c>
       <c r="D25" t="str">
-        <v>ROD. CEL. PM NELSON TRANCHESI, 1730 - ITAQUI, ITAPEVI - SP, 06696-110</v>
+        <v>SAPUCAIA DO SUL, RS</v>
       </c>
       <c r="E25" t="str">
-        <v>ESTR. DOS ALPES, 320 - JARDIM ITAQUITI, BARUERI - SP, 06423-080</v>
+        <v>AV INDUSTRIAL BELGRAF</v>
       </c>
       <c r="F25">
-        <v>8.1</v>
+        <v>36</v>
       </c>
       <c r="G25" t="str">
         <v>(não identificada)</v>
@@ -1926,34 +1950,34 @@
         <v>2264.58</v>
       </c>
       <c r="I25">
-        <v>5.4</v>
+        <v>0</v>
       </c>
       <c r="J25">
-        <v>2269.98</v>
+        <v>2264.58</v>
       </c>
       <c r="K25" t="str">
-        <v>REGIÃO - SUDESTE - ITAPEVI-BARUERI 100KM</v>
+        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
       </c>
       <c r="L25" t="str">
-        <v>exact_route</v>
+        <v>region_band</v>
       </c>
       <c r="M25" t="str">
-        <v>SUDESTE</v>
+        <v>SUL</v>
       </c>
       <c r="N25">
         <v>100</v>
       </c>
       <c r="O25">
-        <v>695.4</v>
+        <v>825.33</v>
       </c>
       <c r="P25">
-        <v>700.8</v>
+        <v>825.33</v>
       </c>
       <c r="Q25">
-        <v>-1569.18</v>
+        <v>-1439.25</v>
       </c>
       <c r="R25" t="str">
-        <v>Rota Exata (SUDESTE + 100km)</v>
+        <v>Sugestão por Proximidade (SUL + 100km)</v>
       </c>
       <c r="S25" t="str">
         <v/>
@@ -1961,22 +1985,22 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>GTM-5071</v>
+        <v>GTM-5074</v>
       </c>
       <c r="B26" t="str">
         <v>Concluída</v>
       </c>
       <c r="C26" t="str">
-        <v>2026-05-20T10:30:00+00:00</v>
+        <v>2026-05-20T09:00:00+00:00</v>
       </c>
       <c r="D26" t="str">
-        <v>FLORIANÓPOLIS, SC</v>
+        <v>R. 20 DE AGOSTO, 1204 - COLONIAL, SAPUCAIA DO SUL - RS, 93212-710</v>
       </c>
       <c r="E26" t="str">
-        <v>FLORIANÓPOLIS, SC</v>
+        <v>BR-116, 7350 - PORTAL DA SERRA, DOIS IRMÃOS - RS, 93950-000</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>31.7</v>
       </c>
       <c r="G26" t="str">
         <v>(não identificada)</v>
@@ -2003,13 +2027,13 @@
         <v>100</v>
       </c>
       <c r="O26">
-        <v>702.08</v>
+        <v>859.17</v>
       </c>
       <c r="P26">
-        <v>702.08</v>
+        <v>859.17</v>
       </c>
       <c r="Q26">
-        <v>-1562.5</v>
+        <v>-1405.41</v>
       </c>
       <c r="R26" t="str">
         <v>Sugestão por Proximidade (SUL + 100km)</v>
@@ -2020,58 +2044,58 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>GTM-5019</v>
+        <v>GTM-5039</v>
       </c>
       <c r="B27" t="str">
-        <v>Concluída</v>
+        <v>Cancelada</v>
       </c>
       <c r="C27" t="str">
-        <v>2026-05-19T10:30:00+00:00</v>
+        <v>2026-05-19T12:00:00+00:00</v>
       </c>
       <c r="D27" t="str">
-        <v>FLORIANÓPOLIS, SC</v>
+        <v>POUSO ALEGRE, MG, 37550-000</v>
       </c>
       <c r="E27" t="str">
-        <v>FLORIANÓPOLIS, SC</v>
+        <v>RAIO 300 KM — DESTINO A DEFINIR</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="G27" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H27">
-        <v>2264.58</v>
+        <v>690</v>
       </c>
       <c r="I27">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="J27">
-        <v>2299.58</v>
+        <v>690</v>
       </c>
       <c r="K27" t="str">
-        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
+        <v>REGIÃO - SUDESTE - RAIO ES 300KM</v>
       </c>
       <c r="L27" t="str">
         <v>region_band</v>
       </c>
       <c r="M27" t="str">
-        <v>SUL</v>
+        <v>SUDESTE</v>
       </c>
       <c r="N27">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="O27">
-        <v>725</v>
+        <v>2070</v>
       </c>
       <c r="P27">
-        <v>760</v>
+        <v>2070</v>
       </c>
       <c r="Q27">
-        <v>-1539.58</v>
+        <v>1380</v>
       </c>
       <c r="R27" t="str">
-        <v>Sugestão por Proximidade (SUL + 100km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 300km)</v>
       </c>
       <c r="S27" t="str">
         <v/>
@@ -2079,58 +2103,58 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>GTM-5160</v>
+        <v>GTM-5123</v>
       </c>
       <c r="B28" t="str">
-        <v>Em Viagem</v>
+        <v>Cancelada</v>
       </c>
       <c r="C28" t="str">
-        <v>2026-05-22T16:30:00+00:00</v>
+        <v>2026-05-21T16:00:00+00:00</v>
       </c>
       <c r="D28" t="str">
-        <v>AV. SEVERO DULLIUS, 90010 - ANCHIETA, PORTO ALEGRE - RS, 90200-310</v>
+        <v>VARGINHA, MG</v>
       </c>
       <c r="E28" t="str">
-        <v>AV. BORGES DE MEDEIROS, 1771 - COLONIAL, SAPUCAIA DO SUL - RS, 93212-110</v>
+        <v>SANTA ROSA, RS</v>
       </c>
       <c r="F28">
-        <v>22.7</v>
+        <v>1479.93</v>
       </c>
       <c r="G28" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H28">
-        <v>2264.58</v>
+        <v>11901.12</v>
       </c>
       <c r="I28">
         <v>0</v>
       </c>
       <c r="J28">
-        <v>2264.58</v>
+        <v>11901.12</v>
       </c>
       <c r="K28" t="str">
-        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
+        <v>REGIÃO - SUDESTE - EXTREMA-PORTO ALEGRE 1464KM</v>
       </c>
       <c r="L28" t="str">
-        <v>region_band</v>
+        <v>region_any_km</v>
       </c>
       <c r="M28" t="str">
-        <v>SUL</v>
+        <v>SUDESTE</v>
       </c>
       <c r="N28">
-        <v>100</v>
+        <v>1500</v>
       </c>
       <c r="O28">
-        <v>726.25</v>
+        <v>10687.2</v>
       </c>
       <c r="P28">
-        <v>726.25</v>
+        <v>10687.2</v>
       </c>
       <c r="Q28">
-        <v>-1538.33</v>
+        <v>-1213.92</v>
       </c>
       <c r="R28" t="str">
-        <v>Sugestão por Proximidade (SUL + 100km)</v>
+        <v>Proximidade Regional (SUDESTE, mais próxima de 1480km)</v>
       </c>
       <c r="S28" t="str">
         <v/>
@@ -2138,58 +2162,58 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>GTM-5161</v>
+        <v>GTM-5057</v>
       </c>
       <c r="B29" t="str">
-        <v>Em Viagem</v>
+        <v>Concluída</v>
       </c>
       <c r="C29" t="str">
-        <v>2026-05-22T16:30:00+00:00</v>
+        <v>2026-05-19T23:30:00+00:00</v>
       </c>
       <c r="D29" t="str">
-        <v>AV. SEVERO DULLIUS, 90010 - ANCHIETA, PORTO ALEGRE - RS, 90200-310</v>
+        <v>ROD. VICE PREF. HERMENEGILDO TONOLI - MEDEIROS, JUNDIAÍ - SP</v>
       </c>
       <c r="E29" t="str">
-        <v>AV. BORGES DE MEDEIROS, 1771 - COLONIAL, SAPUCAIA DO SUL - RS, 93212-110</v>
+        <v>ESTR. MUN. JOSÉ SEDANO - TECHNO PARK, CAMPINAS - SP</v>
       </c>
       <c r="F29">
-        <v>22.7</v>
+        <v>51.9</v>
       </c>
       <c r="G29" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H29">
-        <v>2264.58</v>
+        <v>690</v>
       </c>
       <c r="I29">
-        <v>0</v>
+        <v>12.85</v>
       </c>
       <c r="J29">
-        <v>2264.58</v>
+        <v>702.85</v>
       </c>
       <c r="K29" t="str">
-        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
+        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
       </c>
       <c r="L29" t="str">
         <v>region_band</v>
       </c>
       <c r="M29" t="str">
-        <v>SUL</v>
+        <v>SUDESTE</v>
       </c>
       <c r="N29">
         <v>100</v>
       </c>
       <c r="O29">
-        <v>726.25</v>
+        <v>1824.18</v>
       </c>
       <c r="P29">
-        <v>726.25</v>
+        <v>1837.03</v>
       </c>
       <c r="Q29">
-        <v>-1538.33</v>
+        <v>1134.18</v>
       </c>
       <c r="R29" t="str">
-        <v>Sugestão por Proximidade (SUL + 100km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
       </c>
       <c r="S29" t="str">
         <v/>
@@ -2197,58 +2221,58 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>GTM-5036</v>
+        <v>GTM-5051</v>
       </c>
       <c r="B30" t="str">
         <v>Concluída</v>
       </c>
       <c r="C30" t="str">
-        <v>2026-05-19T10:00:00+00:00</v>
+        <v>2026-05-19T20:30:00+00:00</v>
       </c>
       <c r="D30" t="str">
-        <v>RIO DE JANEIRO, RJ</v>
+        <v>R. VER. GERMANO LUÍS VIÊIRA, 1-1300 - ITAIPAVA, ITAJAÍ - SC, 88316-701</v>
       </c>
       <c r="E30" t="str">
-        <v>RIO DE JANEIRO, RJ</v>
+        <v>AV. CECI, 1900 - JARDIM MUTINGA, BARUERI - SP, 06460-120</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>600.9</v>
       </c>
       <c r="G30" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H30">
-        <v>2264.58</v>
+        <v>3675</v>
       </c>
       <c r="I30">
-        <v>0</v>
+        <v>53.7</v>
       </c>
       <c r="J30">
-        <v>2264.58</v>
+        <v>3728.7</v>
       </c>
       <c r="K30" t="str">
-        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
+        <v>REGIÃO - SUL - RAIO PR 500KM</v>
       </c>
       <c r="L30" t="str">
-        <v>region_band</v>
+        <v>region_any_km</v>
       </c>
       <c r="M30" t="str">
-        <v>SUDESTE</v>
+        <v>SUL</v>
       </c>
       <c r="N30">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="O30">
-        <v>743.17</v>
+        <v>4712.03</v>
       </c>
       <c r="P30">
-        <v>743.17</v>
+        <v>4765.73</v>
       </c>
       <c r="Q30">
-        <v>-1521.41</v>
+        <v>1037.03</v>
       </c>
       <c r="R30" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
+        <v>Proximidade Regional (SUL, mais próxima de 601km)</v>
       </c>
       <c r="S30" t="str">
         <v/>
@@ -2256,58 +2280,58 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>GTM-5030</v>
+        <v>GTM-5069</v>
       </c>
       <c r="B31" t="str">
         <v>Concluída</v>
       </c>
       <c r="C31" t="str">
-        <v>2026-05-19T09:30:00+00:00</v>
+        <v>2026-05-20T08:00:00+00:00</v>
       </c>
       <c r="D31" t="str">
-        <v>R. 20 DE AGOSTO, 1204 - COLONIAL, SAPUCAIA DO SUL - RS, 93212-710</v>
+        <v>ROD. HÉLIO SMIDT, S/N - SETOR 3 - TERMINAL COURIER, GUARULHOS - SP, 07190-100</v>
       </c>
       <c r="E31" t="str">
-        <v>BR-116, 7350 - PORTAL DA SERRA, DOIS IRMÃOS - RS, 93950-000</v>
+        <v>SERRA, ES</v>
       </c>
       <c r="F31">
-        <v>31.7</v>
+        <v>945.9</v>
       </c>
       <c r="G31" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H31">
-        <v>2264.58</v>
+        <v>9920.95</v>
       </c>
       <c r="I31">
-        <v>5.85</v>
+        <v>177.5</v>
       </c>
       <c r="J31">
-        <v>2270.43</v>
+        <v>10098.45</v>
       </c>
       <c r="K31" t="str">
-        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
+        <v>REGIÃO - SUDESTE - LOUVEIRA-APARECIDA DE GOIANIA 946KM</v>
       </c>
       <c r="L31" t="str">
-        <v>region_band</v>
+        <v>region_any_km</v>
       </c>
       <c r="M31" t="str">
-        <v>SUL</v>
+        <v>SUDESTE</v>
       </c>
       <c r="N31">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="O31">
-        <v>778.02</v>
+        <v>10714.15</v>
       </c>
       <c r="P31">
-        <v>783.87</v>
+        <v>10891.65</v>
       </c>
       <c r="Q31">
-        <v>-1486.56</v>
+        <v>793.2</v>
       </c>
       <c r="R31" t="str">
-        <v>Sugestão por Proximidade (SUL + 100km)</v>
+        <v>Proximidade Regional (SUDESTE, mais próxima de 946km)</v>
       </c>
       <c r="S31" t="str">
         <v/>
@@ -2315,58 +2339,58 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>GTM-5155</v>
+        <v>GTM-5150</v>
       </c>
       <c r="B32" t="str">
-        <v>Concluída</v>
+        <v>Em Viagem</v>
       </c>
       <c r="C32" t="str">
-        <v>2026-05-22T09:00:00+00:00</v>
+        <v>2026-05-22T04:00:00+00:00</v>
       </c>
       <c r="D32" t="str">
-        <v>SAPUCAIA DO SUL, RS</v>
+        <v>ESTR. DOS ALPES, 320 - JARDIM ITAQUITI, BARUERI - SP, 06423-080</v>
       </c>
       <c r="E32" t="str">
-        <v>AV INDUSTRIAL BELGRAF</v>
+        <v>BRASÍLIA - PLANO PILOTO, BRASÍLIA - DF</v>
       </c>
       <c r="F32">
-        <v>36</v>
+        <v>1012.7</v>
       </c>
       <c r="G32" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H32">
-        <v>2264.58</v>
+        <v>7990.2</v>
       </c>
       <c r="I32">
         <v>0</v>
       </c>
       <c r="J32">
-        <v>2264.58</v>
+        <v>7990.2</v>
       </c>
       <c r="K32" t="str">
-        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
+        <v>REGIÃO - SUDESTE - GUARULHOS-ANAPOLIS 981KM</v>
       </c>
       <c r="L32" t="str">
-        <v>region_band</v>
+        <v>region_any_km</v>
       </c>
       <c r="M32" t="str">
-        <v>SUL</v>
+        <v>SUDESTE</v>
       </c>
       <c r="N32">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="O32">
-        <v>825.33</v>
+        <v>8722.78</v>
       </c>
       <c r="P32">
-        <v>825.33</v>
+        <v>8722.78</v>
       </c>
       <c r="Q32">
-        <v>-1439.25</v>
+        <v>732.58</v>
       </c>
       <c r="R32" t="str">
-        <v>Sugestão por Proximidade (SUL + 100km)</v>
+        <v>Proximidade Regional (SUDESTE, mais próxima de 1013km)</v>
       </c>
       <c r="S32" t="str">
         <v/>
@@ -2374,58 +2398,58 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>GTM-5074</v>
+        <v>GTM-5112</v>
       </c>
       <c r="B33" t="str">
-        <v>Concluída</v>
+        <v>Recusada</v>
       </c>
       <c r="C33" t="str">
-        <v>2026-05-20T09:00:00+00:00</v>
+        <v>2026-05-21T00:30:00+00:00</v>
       </c>
       <c r="D33" t="str">
-        <v>R. 20 DE AGOSTO, 1204 - COLONIAL, SAPUCAIA DO SUL - RS, 93212-710</v>
+        <v>CAMPINAS, SP</v>
       </c>
       <c r="E33" t="str">
-        <v>BR-116, 7350 - PORTAL DA SERRA, DOIS IRMÃOS - RS, 93950-000</v>
+        <v>LOUVEIRA - SP</v>
       </c>
       <c r="F33">
-        <v>31.7</v>
+        <v>28.2</v>
       </c>
       <c r="G33" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H33">
-        <v>2264.58</v>
+        <v>690</v>
       </c>
       <c r="I33">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J33">
-        <v>2264.58</v>
+        <v>702</v>
       </c>
       <c r="K33" t="str">
-        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
+        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
       </c>
       <c r="L33" t="str">
         <v>region_band</v>
       </c>
       <c r="M33" t="str">
-        <v>SUL</v>
+        <v>SUDESTE</v>
       </c>
       <c r="N33">
         <v>100</v>
       </c>
       <c r="O33">
-        <v>859.17</v>
+        <v>0</v>
       </c>
       <c r="P33">
-        <v>859.17</v>
+        <v>12</v>
       </c>
       <c r="Q33">
-        <v>-1405.41</v>
+        <v>-690</v>
       </c>
       <c r="R33" t="str">
-        <v>Sugestão por Proximidade (SUL + 100km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
       </c>
       <c r="S33" t="str">
         <v/>
@@ -2433,37 +2457,37 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>GTM-5039</v>
+        <v>GTM-5078</v>
       </c>
       <c r="B34" t="str">
-        <v>Cancelada</v>
+        <v>Concluída</v>
       </c>
       <c r="C34" t="str">
-        <v>2026-05-19T12:00:00+00:00</v>
+        <v>2026-05-20T11:05:00+00:00</v>
       </c>
       <c r="D34" t="str">
-        <v>POUSO ALEGRE, MG, 37550-000</v>
+        <v>ESTRADA DOS ALPES, 320 - RESIDENCIAL MORADA DOS LAGOS, JANDIRA - SP, 01250-000</v>
       </c>
       <c r="E34" t="str">
-        <v>RAIO 300 KM — DESTINO A DEFINIR</v>
+        <v>RAIO 200 KM — DESTINO A DEFINIR</v>
       </c>
       <c r="F34">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="G34" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H34">
-        <v>690</v>
+        <v>2070</v>
       </c>
       <c r="I34">
         <v>0</v>
       </c>
       <c r="J34">
-        <v>690</v>
+        <v>2070</v>
       </c>
       <c r="K34" t="str">
-        <v>REGIÃO - SUDESTE - RAIO ES 300KM</v>
+        <v>REGIÃO - SUDESTE - CAJAMAR-RIO DE JANEIRO 200KM</v>
       </c>
       <c r="L34" t="str">
         <v>region_band</v>
@@ -2472,19 +2496,19 @@
         <v>SUDESTE</v>
       </c>
       <c r="N34">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="O34">
-        <v>2070</v>
+        <v>1380</v>
       </c>
       <c r="P34">
-        <v>2070</v>
+        <v>1380</v>
       </c>
       <c r="Q34">
-        <v>1380</v>
+        <v>-690</v>
       </c>
       <c r="R34" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 300km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 200km)</v>
       </c>
       <c r="S34" t="str">
         <v/>
@@ -2492,37 +2516,37 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>GTM-5057</v>
+        <v>GTM-5023</v>
       </c>
       <c r="B35" t="str">
-        <v>Concluída</v>
+        <v>Cancelada</v>
       </c>
       <c r="C35" t="str">
-        <v>2026-05-19T23:30:00+00:00</v>
+        <v>2026-05-19T04:00:00+00:00</v>
       </c>
       <c r="D35" t="str">
-        <v>ROD. VICE PREF. HERMENEGILDO TONOLI - MEDEIROS, JUNDIAÍ - SP</v>
+        <v>ESTRADA DOS ALPES, 320 - RESIDENCIAL MORADA DOS LAGOS, JANDIRA - SP, 01250-000</v>
       </c>
       <c r="E35" t="str">
-        <v>ESTR. MUN. JOSÉ SEDANO - TECHNO PARK, CAMPINAS - SP</v>
+        <v>RAIO 200 KM — DESTINO A DEFINIR</v>
       </c>
       <c r="F35">
-        <v>51.9</v>
+        <v>200</v>
       </c>
       <c r="G35" t="str">
-        <v>(não identificada)</v>
+        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
       </c>
       <c r="H35">
         <v>690</v>
       </c>
       <c r="I35">
-        <v>12.85</v>
+        <v>0</v>
       </c>
       <c r="J35">
-        <v>702.85</v>
+        <v>690</v>
       </c>
       <c r="K35" t="str">
-        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
+        <v>REGIÃO - SUDESTE - CAJAMAR-RIO DE JANEIRO 200KM</v>
       </c>
       <c r="L35" t="str">
         <v>region_band</v>
@@ -2531,19 +2555,19 @@
         <v>SUDESTE</v>
       </c>
       <c r="N35">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="O35">
-        <v>1824.18</v>
+        <v>1380</v>
       </c>
       <c r="P35">
-        <v>1837.03</v>
+        <v>1380</v>
       </c>
       <c r="Q35">
-        <v>1134.18</v>
+        <v>690</v>
       </c>
       <c r="R35" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 200km)</v>
       </c>
       <c r="S35" t="str">
         <v/>
@@ -2551,37 +2575,37 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>GTM-5112</v>
+        <v>GTM-5116</v>
       </c>
       <c r="B36" t="str">
-        <v>Recusada</v>
+        <v>Cancelada</v>
       </c>
       <c r="C36" t="str">
-        <v>2026-05-21T00:30:00+00:00</v>
+        <v>2026-05-21T05:00:00+00:00</v>
       </c>
       <c r="D36" t="str">
-        <v>CAMPINAS, SP</v>
+        <v>ESTRADA DOS ALPES, 320 - RESIDENCIAL MORADA DOS LAGOS, JANDIRA - SP, 01250-000</v>
       </c>
       <c r="E36" t="str">
-        <v>LOUVEIRA - SP</v>
+        <v>RAIO 200 KM — DESTINO A DEFINIR</v>
       </c>
       <c r="F36">
-        <v>28.2</v>
+        <v>200</v>
       </c>
       <c r="G36" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H36">
-        <v>690</v>
+        <v>2070</v>
       </c>
       <c r="I36">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J36">
-        <v>702</v>
+        <v>2070</v>
       </c>
       <c r="K36" t="str">
-        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
+        <v>REGIÃO - SUDESTE - CAJAMAR-RIO DE JANEIRO 200KM</v>
       </c>
       <c r="L36" t="str">
         <v>region_band</v>
@@ -2590,19 +2614,19 @@
         <v>SUDESTE</v>
       </c>
       <c r="N36">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="O36">
-        <v>0</v>
+        <v>1416.25</v>
       </c>
       <c r="P36">
-        <v>12</v>
+        <v>1416.25</v>
       </c>
       <c r="Q36">
-        <v>-690</v>
+        <v>-653.75</v>
       </c>
       <c r="R36" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 200km)</v>
       </c>
       <c r="S36" t="str">
         <v/>
@@ -2610,58 +2634,58 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>GTM-5078</v>
+        <v>GTM-5070</v>
       </c>
       <c r="B37" t="str">
         <v>Concluída</v>
       </c>
       <c r="C37" t="str">
-        <v>2026-05-20T11:05:00+00:00</v>
+        <v>2026-05-20T10:00:00+00:00</v>
       </c>
       <c r="D37" t="str">
-        <v>ESTRADA DOS ALPES, 320 - RESIDENCIAL MORADA DOS LAGOS, JANDIRA - SP, 01250-000</v>
+        <v>ROD. HÉLIO SMIDT, S/N - SETOR 3 - TERMINAL COURIER, GUARULHOS - SP, 07190-100</v>
       </c>
       <c r="E37" t="str">
-        <v>RAIO 200 KM — DESTINO A DEFINIR</v>
+        <v>SERRA, ES</v>
       </c>
       <c r="F37">
-        <v>200</v>
+        <v>945.9</v>
       </c>
       <c r="G37" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H37">
-        <v>2070</v>
+        <v>9628.53</v>
       </c>
       <c r="I37">
         <v>0</v>
       </c>
       <c r="J37">
-        <v>2070</v>
+        <v>9628.53</v>
       </c>
       <c r="K37" t="str">
-        <v>REGIÃO - SUDESTE - CAJAMAR-RIO DE JANEIRO 200KM</v>
+        <v>REGIÃO - SUDESTE - LOUVEIRA-APARECIDA DE GOIANIA 946KM</v>
       </c>
       <c r="L37" t="str">
-        <v>region_band</v>
+        <v>region_any_km</v>
       </c>
       <c r="M37" t="str">
         <v>SUDESTE</v>
       </c>
       <c r="N37">
-        <v>200</v>
+        <v>900</v>
       </c>
       <c r="O37">
-        <v>1380</v>
+        <v>10244.23</v>
       </c>
       <c r="P37">
-        <v>1380</v>
+        <v>10244.23</v>
       </c>
       <c r="Q37">
-        <v>-690</v>
+        <v>615.7</v>
       </c>
       <c r="R37" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 200km)</v>
+        <v>Proximidade Regional (SUDESTE, mais próxima de 946km)</v>
       </c>
       <c r="S37" t="str">
         <v/>
@@ -2669,37 +2693,37 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>GTM-5023</v>
+        <v>GTM-5152</v>
       </c>
       <c r="B38" t="str">
-        <v>Cancelada</v>
+        <v>Concluída</v>
       </c>
       <c r="C38" t="str">
-        <v>2026-05-19T04:00:00+00:00</v>
+        <v>2026-05-22T08:00:00+00:00</v>
       </c>
       <c r="D38" t="str">
-        <v>ESTRADA DOS ALPES, 320 - RESIDENCIAL MORADA DOS LAGOS, JANDIRA - SP, 01250-000</v>
+        <v>ESTR. DOS ALPES, 320 - JARDIM ITAQUITI, BARUERI - SP, 06423-080</v>
       </c>
       <c r="E38" t="str">
-        <v>RAIO 200 KM — DESTINO A DEFINIR</v>
+        <v>SÃO PAULO, SP</v>
       </c>
       <c r="F38">
-        <v>200</v>
+        <v>38.2</v>
       </c>
       <c r="G38" t="str">
-        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
+        <v>(não identificada)</v>
       </c>
       <c r="H38">
-        <v>690</v>
+        <v>1378.75</v>
       </c>
       <c r="I38">
         <v>0</v>
       </c>
       <c r="J38">
-        <v>690</v>
+        <v>1378.75</v>
       </c>
       <c r="K38" t="str">
-        <v>REGIÃO - SUDESTE - CAJAMAR-RIO DE JANEIRO 200KM</v>
+        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
       </c>
       <c r="L38" t="str">
         <v>region_band</v>
@@ -2708,19 +2732,19 @@
         <v>SUDESTE</v>
       </c>
       <c r="N38">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="O38">
-        <v>1380</v>
+        <v>943.75</v>
       </c>
       <c r="P38">
-        <v>1380</v>
+        <v>943.75</v>
       </c>
       <c r="Q38">
-        <v>690</v>
+        <v>-435</v>
       </c>
       <c r="R38" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 200km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
       </c>
       <c r="S38" t="str">
         <v/>
@@ -2728,37 +2752,37 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>GTM-5116</v>
+        <v>GTM-5044</v>
       </c>
       <c r="B39" t="str">
-        <v>Cancelada</v>
+        <v>Concluída</v>
       </c>
       <c r="C39" t="str">
-        <v>2026-05-21T05:00:00+00:00</v>
+        <v>2026-05-19T15:00:00+00:00</v>
       </c>
       <c r="D39" t="str">
-        <v>ESTRADA DOS ALPES, 320 - RESIDENCIAL MORADA DOS LAGOS, JANDIRA - SP, 01250-000</v>
+        <v>ROD. HÉLIO SMIDT, S/N - SETOR 3 - TERMINAL COURIER, GUARULHOS - SP, 07190-100</v>
       </c>
       <c r="E39" t="str">
-        <v>RAIO 200 KM — DESTINO A DEFINIR</v>
+        <v>JANDIRA, SP</v>
       </c>
       <c r="F39">
-        <v>200</v>
+        <v>55.7</v>
       </c>
       <c r="G39" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H39">
-        <v>2070</v>
+        <v>1040.42</v>
       </c>
       <c r="I39">
         <v>0</v>
       </c>
       <c r="J39">
-        <v>2070</v>
+        <v>1040.42</v>
       </c>
       <c r="K39" t="str">
-        <v>REGIÃO - SUDESTE - CAJAMAR-RIO DE JANEIRO 200KM</v>
+        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
       </c>
       <c r="L39" t="str">
         <v>region_band</v>
@@ -2767,19 +2791,19 @@
         <v>SUDESTE</v>
       </c>
       <c r="N39">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="O39">
-        <v>1416.25</v>
+        <v>690</v>
       </c>
       <c r="P39">
-        <v>1416.25</v>
+        <v>690</v>
       </c>
       <c r="Q39">
-        <v>-653.75</v>
+        <v>-350.42</v>
       </c>
       <c r="R39" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 200km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
       </c>
       <c r="S39" t="str">
         <v/>
@@ -2787,34 +2811,34 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>GTM-5152</v>
+        <v>GTM-5040</v>
       </c>
       <c r="B40" t="str">
         <v>Concluída</v>
       </c>
       <c r="C40" t="str">
-        <v>2026-05-22T08:00:00+00:00</v>
+        <v>2026-05-20T00:00:00+00:00</v>
       </c>
       <c r="D40" t="str">
-        <v>ESTR. DOS ALPES, 320 - JARDIM ITAQUITI, BARUERI - SP, 06423-080</v>
+        <v>ROD. HÉLIO SMIDT, S/N - SETOR 3 - TERMINAL COURIER, GUARULHOS - SP, 07190-100</v>
       </c>
       <c r="E40" t="str">
-        <v>SÃO PAULO, SP</v>
+        <v>BARUERI, SP</v>
       </c>
       <c r="F40">
-        <v>38.2</v>
+        <v>51.9</v>
       </c>
       <c r="G40" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H40">
-        <v>1378.75</v>
+        <v>965.5</v>
       </c>
       <c r="I40">
-        <v>0</v>
+        <v>18.2</v>
       </c>
       <c r="J40">
-        <v>1378.75</v>
+        <v>983.7</v>
       </c>
       <c r="K40" t="str">
         <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
@@ -2829,13 +2853,13 @@
         <v>100</v>
       </c>
       <c r="O40">
-        <v>943.75</v>
+        <v>708.2</v>
       </c>
       <c r="P40">
-        <v>943.75</v>
+        <v>726.4</v>
       </c>
       <c r="Q40">
-        <v>-435</v>
+        <v>-257.3</v>
       </c>
       <c r="R40" t="str">
         <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
@@ -2846,43 +2870,43 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>GTM-5044</v>
+        <v>GTM-5128</v>
       </c>
       <c r="B41" t="str">
         <v>Concluída</v>
       </c>
       <c r="C41" t="str">
-        <v>2026-05-19T15:00:00+00:00</v>
+        <v>2026-05-21T17:20:00+00:00</v>
       </c>
       <c r="D41" t="str">
-        <v>ROD. HÉLIO SMIDT, S/N - SETOR 3 - TERMINAL COURIER, GUARULHOS - SP, 07190-100</v>
+        <v>AV. ROCHA POMBO - ÁGUAS BELAS, SÃO JOSÉ DOS PINHAIS - PR, 83010-900</v>
       </c>
       <c r="E41" t="str">
-        <v>JANDIRA, SP</v>
+        <v>R. FRANCISCO MUNÕZ MADRID, 625 - ROSEIRA DE SÃO SEBASTIÃO, SÃO JOSÉ DOS PINHAIS - PR, 83070-010</v>
       </c>
       <c r="F41">
-        <v>55.7</v>
+        <v>100</v>
       </c>
       <c r="G41" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H41">
-        <v>1040.42</v>
+        <v>938.4</v>
       </c>
       <c r="I41">
         <v>0</v>
       </c>
       <c r="J41">
-        <v>1040.42</v>
+        <v>938.4</v>
       </c>
       <c r="K41" t="str">
-        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
+        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
       </c>
       <c r="L41" t="str">
         <v>region_band</v>
       </c>
       <c r="M41" t="str">
-        <v>SUDESTE</v>
+        <v>SUL</v>
       </c>
       <c r="N41">
         <v>100</v>
@@ -2894,10 +2918,10 @@
         <v>690</v>
       </c>
       <c r="Q41">
-        <v>-350.42</v>
+        <v>-248.4</v>
       </c>
       <c r="R41" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
+        <v>Sugestão por Proximidade (SUL + 100km)</v>
       </c>
       <c r="S41" t="str">
         <v/>
@@ -2905,58 +2929,58 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>GTM-5040</v>
+        <v>GTM-5135</v>
       </c>
       <c r="B42" t="str">
         <v>Concluída</v>
       </c>
       <c r="C42" t="str">
-        <v>2026-05-20T00:00:00+00:00</v>
+        <v>2026-05-21T21:40:00+00:00</v>
       </c>
       <c r="D42" t="str">
-        <v>ROD. HÉLIO SMIDT, S/N - SETOR 3 - TERMINAL COURIER, GUARULHOS - SP, 07190-100</v>
+        <v>R. VER. GERMANO LUÍS VIÊIRA - ITAIPAVA, ITAJAÍ - SC</v>
       </c>
       <c r="E42" t="str">
-        <v>BARUERI, SP</v>
+        <v>AV. CECI - TAMBORÉ, BARUERI - SP, 06460-120</v>
       </c>
       <c r="F42">
-        <v>51.9</v>
+        <v>600</v>
       </c>
       <c r="G42" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H42">
-        <v>965.5</v>
+        <v>3989.17</v>
       </c>
       <c r="I42">
-        <v>18.2</v>
+        <v>0</v>
       </c>
       <c r="J42">
-        <v>983.7</v>
+        <v>3989.17</v>
       </c>
       <c r="K42" t="str">
-        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
+        <v>REGIÃO - SUL - RAIO PR 500KM</v>
       </c>
       <c r="L42" t="str">
-        <v>region_band</v>
+        <v>region_any_km</v>
       </c>
       <c r="M42" t="str">
-        <v>SUDESTE</v>
+        <v>SUL</v>
       </c>
       <c r="N42">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="O42">
-        <v>708.2</v>
+        <v>3764.17</v>
       </c>
       <c r="P42">
-        <v>726.4</v>
+        <v>3764.17</v>
       </c>
       <c r="Q42">
-        <v>-257.3</v>
+        <v>-225</v>
       </c>
       <c r="R42" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
+        <v>Proximidade Regional (SUL, mais próxima de 600km)</v>
       </c>
       <c r="S42" t="str">
         <v/>
@@ -2964,37 +2988,37 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>GTM-5128</v>
+        <v>GTM-5127</v>
       </c>
       <c r="B43" t="str">
         <v>Concluída</v>
       </c>
       <c r="C43" t="str">
-        <v>2026-05-21T17:20:00+00:00</v>
+        <v>2026-05-21T16:00:00+00:00</v>
       </c>
       <c r="D43" t="str">
-        <v>AV. ROCHA POMBO - ÁGUAS BELAS, SÃO JOSÉ DOS PINHAIS - PR, 83010-900</v>
+        <v>AV. BORGES DE MEDEIROS, 1771 - COLONIAL, SAPUCAIA DO SUL - RS, 93212-110</v>
       </c>
       <c r="E43" t="str">
-        <v>R. FRANCISCO MUNÕZ MADRID, 625 - ROSEIRA DE SÃO SEBASTIÃO, SÃO JOSÉ DOS PINHAIS - PR, 83070-010</v>
+        <v>RAIO 500 KM — DESTINO A DEFINIR</v>
       </c>
       <c r="F43">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="G43" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H43">
-        <v>938.4</v>
+        <v>3675</v>
       </c>
       <c r="I43">
         <v>0</v>
       </c>
       <c r="J43">
-        <v>938.4</v>
+        <v>3675</v>
       </c>
       <c r="K43" t="str">
-        <v>REGIÃO - SUL - DISTRIBUIÇÃO PR 100KM</v>
+        <v>REGIÃO - SUL - RAIO PR 500KM</v>
       </c>
       <c r="L43" t="str">
         <v>region_band</v>
@@ -3003,19 +3027,19 @@
         <v>SUL</v>
       </c>
       <c r="N43">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="O43">
-        <v>690</v>
+        <v>3450</v>
       </c>
       <c r="P43">
-        <v>690</v>
+        <v>3450</v>
       </c>
       <c r="Q43">
-        <v>-248.4</v>
+        <v>-225</v>
       </c>
       <c r="R43" t="str">
-        <v>Sugestão por Proximidade (SUL + 100km)</v>
+        <v>Sugestão por Proximidade (SUL + 500km)</v>
       </c>
       <c r="S43" t="str">
         <v/>
@@ -3023,58 +3047,58 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>GTM-5127</v>
+        <v>GTM-5138</v>
       </c>
       <c r="B44" t="str">
         <v>Concluída</v>
       </c>
       <c r="C44" t="str">
-        <v>2026-05-21T16:00:00+00:00</v>
+        <v>2026-05-22T00:00:00+00:00</v>
       </c>
       <c r="D44" t="str">
-        <v>AV. BORGES DE MEDEIROS, 1771 - COLONIAL, SAPUCAIA DO SUL - RS, 93212-110</v>
+        <v>ROD. FERNÃO DIAS, KM 947 - PIRES, EXTREMA - MG, 37640-000</v>
       </c>
       <c r="E44" t="str">
-        <v>RAIO 500 KM — DESTINO A DEFINIR</v>
+        <v>RAIO 400 KM — DESTINO A DEFINIR</v>
       </c>
       <c r="F44">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="G44" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H44">
-        <v>3675</v>
+        <v>2920</v>
       </c>
       <c r="I44">
         <v>0</v>
       </c>
       <c r="J44">
-        <v>3675</v>
+        <v>2920</v>
       </c>
       <c r="K44" t="str">
-        <v>REGIÃO - SUL - RAIO PR 500KM</v>
+        <v>REGIÃO - SUDESTE - RAIO ES 400KM</v>
       </c>
       <c r="L44" t="str">
         <v>region_band</v>
       </c>
       <c r="M44" t="str">
-        <v>SUL</v>
+        <v>SUDESTE</v>
       </c>
       <c r="N44">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="O44">
-        <v>3450</v>
+        <v>2760</v>
       </c>
       <c r="P44">
-        <v>3450</v>
+        <v>2760</v>
       </c>
       <c r="Q44">
-        <v>-225</v>
+        <v>-160</v>
       </c>
       <c r="R44" t="str">
-        <v>Sugestão por Proximidade (SUL + 500km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 400km)</v>
       </c>
       <c r="S44" t="str">
         <v/>
@@ -3082,37 +3106,37 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>GTM-5138</v>
+        <v>GTM-5151</v>
       </c>
       <c r="B45" t="str">
-        <v>Concluída</v>
+        <v>Cancelada</v>
       </c>
       <c r="C45" t="str">
-        <v>2026-05-22T00:00:00+00:00</v>
+        <v>2026-05-22T04:00:00+00:00</v>
       </c>
       <c r="D45" t="str">
-        <v>ROD. FERNÃO DIAS, KM 947 - PIRES, EXTREMA - MG, 37640-000</v>
+        <v>ESTR. DOS ALPES, 320 - JARDIM ITAQUITI, BARUERI - SP, 06423-080</v>
       </c>
       <c r="E45" t="str">
-        <v>RAIO 400 KM — DESTINO A DEFINIR</v>
+        <v>RAIO 200 KM — DESTINO A DEFINIR</v>
       </c>
       <c r="F45">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="G45" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H45">
-        <v>2920</v>
+        <v>1538.7</v>
       </c>
       <c r="I45">
         <v>0</v>
       </c>
       <c r="J45">
-        <v>2920</v>
+        <v>1538.7</v>
       </c>
       <c r="K45" t="str">
-        <v>REGIÃO - SUDESTE - RAIO ES 400KM</v>
+        <v>REGIÃO - SUDESTE - CAJAMAR-RIO DE JANEIRO 200KM</v>
       </c>
       <c r="L45" t="str">
         <v>region_band</v>
@@ -3121,19 +3145,19 @@
         <v>SUDESTE</v>
       </c>
       <c r="N45">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="O45">
-        <v>2760</v>
+        <v>1380</v>
       </c>
       <c r="P45">
-        <v>2760</v>
+        <v>1380</v>
       </c>
       <c r="Q45">
-        <v>-160</v>
+        <v>-158.7</v>
       </c>
       <c r="R45" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 400km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 200km)</v>
       </c>
       <c r="S45" t="str">
         <v/>
@@ -3141,13 +3165,13 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>GTM-5151</v>
+        <v>GTM-5058</v>
       </c>
       <c r="B46" t="str">
-        <v>Cancelada</v>
+        <v>Concluída</v>
       </c>
       <c r="C46" t="str">
-        <v>2026-05-22T04:00:00+00:00</v>
+        <v>2026-05-20T01:00:00+00:00</v>
       </c>
       <c r="D46" t="str">
         <v>ESTR. DOS ALPES, 320 - JARDIM ITAQUITI, BARUERI - SP, 06423-080</v>
@@ -3200,37 +3224,37 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>GTM-5058</v>
+        <v>GTM-5024</v>
       </c>
       <c r="B47" t="str">
         <v>Concluída</v>
       </c>
       <c r="C47" t="str">
-        <v>2026-05-20T01:00:00+00:00</v>
+        <v>2026-05-19T10:30:00+00:00</v>
       </c>
       <c r="D47" t="str">
-        <v>ESTR. DOS ALPES, 320 - JARDIM ITAQUITI, BARUERI - SP, 06423-080</v>
+        <v>R. 4E - CIVIT II, SERRA - ES, 29168-082</v>
       </c>
       <c r="E47" t="str">
-        <v>RAIO 200 KM — DESTINO A DEFINIR</v>
+        <v>RAIO 300 KM — DESTINO A DEFINIR</v>
       </c>
       <c r="F47">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="G47" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H47">
-        <v>1538.7</v>
+        <v>2190</v>
       </c>
       <c r="I47">
         <v>0</v>
       </c>
       <c r="J47">
-        <v>1538.7</v>
+        <v>2190</v>
       </c>
       <c r="K47" t="str">
-        <v>REGIÃO - SUDESTE - CAJAMAR-RIO DE JANEIRO 200KM</v>
+        <v>REGIÃO - SUDESTE - RAIO ES 300KM</v>
       </c>
       <c r="L47" t="str">
         <v>region_band</v>
@@ -3239,19 +3263,19 @@
         <v>SUDESTE</v>
       </c>
       <c r="N47">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="O47">
-        <v>1380</v>
+        <v>2070</v>
       </c>
       <c r="P47">
-        <v>1380</v>
+        <v>2070</v>
       </c>
       <c r="Q47">
-        <v>-158.7</v>
+        <v>-120</v>
       </c>
       <c r="R47" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 200km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 300km)</v>
       </c>
       <c r="S47" t="str">
         <v/>
@@ -3259,37 +3283,37 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>GTM-5024</v>
+        <v>GTM-5117</v>
       </c>
       <c r="B48" t="str">
         <v>Concluída</v>
       </c>
       <c r="C48" t="str">
-        <v>2026-05-19T10:30:00+00:00</v>
+        <v>2026-05-21T08:00:00+00:00</v>
       </c>
       <c r="D48" t="str">
-        <v>R. 4E - CIVIT II, SERRA - ES, 29168-082</v>
+        <v>JANDIRA, SP</v>
       </c>
       <c r="E48" t="str">
-        <v>RAIO 300 KM — DESTINO A DEFINIR</v>
+        <v>SÃO PAULO, SP</v>
       </c>
       <c r="F48">
-        <v>300</v>
+        <v>37.9</v>
       </c>
       <c r="G48" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H48">
-        <v>2190</v>
+        <v>796.33</v>
       </c>
       <c r="I48">
         <v>0</v>
       </c>
       <c r="J48">
-        <v>2190</v>
+        <v>796.33</v>
       </c>
       <c r="K48" t="str">
-        <v>REGIÃO - SUDESTE - RAIO ES 300KM</v>
+        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
       </c>
       <c r="L48" t="str">
         <v>region_band</v>
@@ -3298,19 +3322,19 @@
         <v>SUDESTE</v>
       </c>
       <c r="N48">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="O48">
-        <v>2070</v>
+        <v>690</v>
       </c>
       <c r="P48">
-        <v>2070</v>
+        <v>690</v>
       </c>
       <c r="Q48">
-        <v>-120</v>
+        <v>-106.33</v>
       </c>
       <c r="R48" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 300km)</v>
+        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
       </c>
       <c r="S48" t="str">
         <v/>
@@ -3318,58 +3342,58 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>GTM-5117</v>
+        <v>GTM-5134</v>
       </c>
       <c r="B49" t="str">
         <v>Concluída</v>
       </c>
       <c r="C49" t="str">
-        <v>2026-05-21T08:00:00+00:00</v>
+        <v>2026-05-21T21:40:00+00:00</v>
       </c>
       <c r="D49" t="str">
-        <v>JANDIRA, SP</v>
+        <v>R. VER. GERMANO LUÍS VIÊIRA - ITAIPAVA, ITAJAÍ - SC</v>
       </c>
       <c r="E49" t="str">
-        <v>SÃO PAULO, SP</v>
+        <v>AV. CECI - TAMBORÉ, BARUERI - SP, 06460-120</v>
       </c>
       <c r="F49">
-        <v>37.9</v>
+        <v>600</v>
       </c>
       <c r="G49" t="str">
         <v>(não identificada)</v>
       </c>
       <c r="H49">
-        <v>796.33</v>
+        <v>3675</v>
       </c>
       <c r="I49">
         <v>0</v>
       </c>
       <c r="J49">
-        <v>796.33</v>
+        <v>3675</v>
       </c>
       <c r="K49" t="str">
-        <v>REGIÃO - SUDESTE - BARUERI-CAJAMAR 100KM</v>
+        <v>REGIÃO - SUL - RAIO PR 500KM</v>
       </c>
       <c r="L49" t="str">
-        <v>region_band</v>
+        <v>region_any_km</v>
       </c>
       <c r="M49" t="str">
-        <v>SUDESTE</v>
+        <v>SUL</v>
       </c>
       <c r="N49">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="O49">
-        <v>690</v>
+        <v>3769</v>
       </c>
       <c r="P49">
-        <v>690</v>
+        <v>3769</v>
       </c>
       <c r="Q49">
-        <v>-106.33</v>
+        <v>94</v>
       </c>
       <c r="R49" t="str">
-        <v>Sugestão por Proximidade (SUDESTE + 100km)</v>
+        <v>Proximidade Regional (SUL, mais próxima de 600km)</v>
       </c>
       <c r="S49" t="str">
         <v/>

</xml_diff>